<commit_message>
added same group loop logic
</commit_message>
<xml_diff>
--- a/samples/request_list.xlsx
+++ b/samples/request_list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
   <si>
     <t>Security Group</t>
   </si>
@@ -34,7 +34,7 @@
     <t>Put</t>
   </si>
   <si>
-    <t>ISSG_INT012_Sreenath</t>
+    <t>ISSG_INT_Final_CCW_Outbound_SREENATH_ASN</t>
   </si>
   <si>
     <t xml:space="preserve">Worker Data: Compensation Grade
@@ -47,7 +47,11 @@
     <t>N</t>
   </si>
   <si>
-    <t>Worker Data: Compensation Management</t>
+    <t>ISSG_INT012_Sreenath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Job Profile: Manage Job Profile Events</t>
   </si>
   <si>
     <t>ISSG_INT001_SREE_Practice</t>
@@ -483,10 +487,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>8</v>
@@ -503,10 +507,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
made sure for R-Tenant
</commit_message>
<xml_diff>
--- a/samples/request_list.xlsx
+++ b/samples/request_list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="13">
   <si>
     <t>Security Group</t>
   </si>
@@ -41,13 +41,10 @@
 </t>
   </si>
   <si>
+    <t>N</t>
+  </si>
+  <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>ISSG_INT012_Sreenath</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -76,7 +73,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -476,21 +473,21 @@
         <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>8</v>
@@ -507,22 +504,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>